<commit_message>
chore: add sex, age and GCS into database
</commit_message>
<xml_diff>
--- a/oxytcmri/test-data/subjects_list.xlsx
+++ b/oxytcmri/test-data/subjects_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/PSL/NextCloud Leviia/01 - Projets/IRM Oxy-TC/oxytcmri/oxytcmri/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4B7A86B-EDB7-594F-BF8D-CFF959F1C1B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54B3BDA2-404C-3C45-919B-E473AF289C86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="480" yWindow="1000" windowWidth="25040" windowHeight="14400" xr2:uid="{285C4748-E489-DC43-ADA7-3AB202FEEF15}"/>
   </bookViews>
@@ -505,7 +505,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F4D29C-63CC-6F4C-A1AC-98FE743175FC}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -525,7 +524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -536,7 +535,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -547,7 +546,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -613,7 +612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -635,7 +634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -646,7 +645,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -657,7 +656,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -668,7 +667,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -690,7 +689,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>24</v>
       </c>
@@ -701,7 +700,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -712,7 +711,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>26</v>
       </c>
@@ -723,7 +722,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -779,13 +778,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C24" xr:uid="{C2F4D29C-63CC-6F4C-A1AC-98FE743175FC}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Patient"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C24" xr:uid="{C2F4D29C-63CC-6F4C-A1AC-98FE743175FC}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>